<commit_message>
Translate all labels to English, switch figures to rates per 1,000 LB
- All figure labels, axis titles, legends in English
- Race/colour: White, Black, Mixed-race, Asian, Indigenous
- Regions: North, Northeast, Southeast, South, Central-West
- IVS categories: Very low, Low, Medium, High, Very high
- Fig1 now shows rates per 1,000 live births (not absolute cases)
- Fig2 shows rates by region (not absolute cases)
- Absolute cases moved to supplementary (FigS1)
- Manuscript Word regenerated with new figures

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/R_analysis/output/supplementary/Dicionario_Variaveis.xlsx
+++ b/R_analysis/output/supplementary/Dicionario_Variaveis.xlsx
@@ -384,7 +384,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Ano de notificação</t>
+          <t>Year of notification</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -494,7 +494,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Tipo: Gestacional ou Congênita</t>
+          <t>Tipo: Gestational ou Congenital</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">

</xml_diff>

<commit_message>
Final cleanup: all English, corrected references, rates throughout
- All remaining Portuguese labels translated to English
- Variable dictionary in English
- 6 references corrected per PubMed verification
- Joinpoint figure uses rates (not absolute cases)
- Fig1 panel: rate/1000 LB + incidence/100k inhabitants
- Map panel: rates + LISA combined
- Manuscript Word regenerated with corrected references

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/R_analysis/output/supplementary/Dicionario_Variaveis.xlsx
+++ b/R_analysis/output/supplementary/Dicionario_Variaveis.xlsx
@@ -362,12 +362,12 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Descricao</t>
+          <t>Description</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Fonte</t>
+          <t>Source</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -406,7 +406,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Código IBGE do município (6 dígitos)</t>
+          <t>IBGE municipality code (6 digits)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -428,7 +428,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Código da UF (2 dígitos)</t>
+          <t>State code (2 digits)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -450,12 +450,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Macrorregião do Brasil</t>
+          <t>Macro-region of Brazil</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Derivada</t>
+          <t>Derived</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -472,7 +472,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Raça/cor (autorreferida/mãe)</t>
+          <t>Race/colour (self-reported/maternal)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -494,12 +494,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Tipo: Gestational ou Congenital</t>
+          <t>Type: Gestational or Congenital</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Derivada</t>
+          <t>Derived</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -516,7 +516,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Número de casos notificados</t>
+          <t>Number of notified cases</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -538,7 +538,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Nascidos vivos (denominador)</t>
+          <t>Live births (denominator)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -560,12 +560,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Taxa por 1.000 nascidos vivos (bruta)</t>
+          <t>Crude rate per 1,000 live births</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Calculada</t>
+          <t>Calculated</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -582,12 +582,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Taxa suavizada por Bayes empírico (/1.000 NV)</t>
+          <t>Empirical Bayes smoothed rate (/1,000 LB)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Calculada (Bayes empírico)</t>
+          <t>Calculated (Empirical Bayes)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -604,7 +604,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Índice de Vulnerabilidade Social (IPEA) — geral</t>
+          <t>Social Vulnerability Index (IPEA) — overall</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -626,7 +626,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>IVS — dimensão Infraestrutura Urbana</t>
+          <t>IVS — Urban Infrastructure dimension</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -648,7 +648,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>IVS — dimensão Capital Humano</t>
+          <t>IVS — Human Capital dimension</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -670,7 +670,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>IVS — dimensão Renda e Trabalho</t>
+          <t>IVS — Income and Labour dimension</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -692,12 +692,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Categoria de IVS (muito baixa a muito alta)</t>
+          <t>IVS category (very low to very high)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Derivada do IVS</t>
+          <t>Derived from IVS</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -714,12 +714,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Quintil de IVS (1=menos vulnerável, 5=mais vulnerável)</t>
+          <t>IVS quintile (1=least vulnerable, 5=most vulnerable)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Derivada do IVS</t>
+          <t>Derived from IVS</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -736,12 +736,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Classificação LISA (High-High, Low-Low, etc.)</t>
+          <t>LISA classification (High-High, Low-Low, etc.)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Calculada (spdep)</t>
+          <t>Calculated (spdep)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -758,12 +758,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Razão sífilis congênita / sífilis gestacional</t>
+          <t>Congenital/gestational syphilis ratio</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Calculada</t>
+          <t>Calculated</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">

</xml_diff>